<commit_message>
annual market twosides turnover
</commit_message>
<xml_diff>
--- a/rqalpha/mod/rqalpha_mod_sys_analyser/report/templates/summary.xlsx
+++ b/rqalpha/mod/rqalpha_mod_sys_analyser/report/templates/summary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Code\ricequant\rqalpha\rqalpha\mod\rqalpha_mod_sys_analyser\report\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cuiziqi/Workspace/RQSDK/rqalpha/rqalpha/mod/rqalpha_mod_sys_analyser/report/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40DD12C8-EBB8-4C89-88FD-1F4BF1334802}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{658871ED-7D5C-E04F-AEAB-1F0807668FF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="44760" yWindow="3690" windowWidth="28800" windowHeight="15435" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="概览" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="月度收益" sheetId="3" r:id="rId3"/>
     <sheet name="月度超额收益（几何）" sheetId="4" r:id="rId4"/>
     <sheet name="个股权重" sheetId="5" r:id="rId5"/>
-    <sheet name="压力测试" sheetId="7" r:id="rId6"/>
+    <sheet name="压力测试" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="daily__date_count">COUNTA(个股权重!$A:$A)-1</definedName>
@@ -29,12 +29,12 @@
     <definedName name="daily__weight_max">OFFSET(个股权重!$I$2,0,0,daily__date_count)</definedName>
     <definedName name="daily__weight_mean">OFFSET(个股权重!$C$2,0,0,daily__date_count)</definedName>
   </definedNames>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="177">
   <si>
     <t>策略名称</t>
   </si>
@@ -108,10 +108,10 @@
     <t>#unit_net_value#</t>
   </si>
   <si>
-    <t>份额</t>
-  </si>
-  <si>
-    <t>#units#</t>
+    <t>年化双边换手倍数</t>
+  </si>
+  <si>
+    <t>#annualized_twoside_turnover#</t>
   </si>
   <si>
     <t>换手率</t>
@@ -357,6 +357,18 @@
     <t>超额收益率（几何）</t>
   </si>
   <si>
+    <t>收益最大回撤</t>
+  </si>
+  <si>
+    <t>最大回撤持续时间</t>
+  </si>
+  <si>
+    <t>超额最大回撤（几何）</t>
+  </si>
+  <si>
+    <t>超额最大回撤持续时间</t>
+  </si>
+  <si>
     <t>超额收益年化波动率</t>
   </si>
   <si>
@@ -541,115 +553,19 @@
   </si>
   <si>
     <t>名称（标题）</t>
+  </si>
+  <si>
+    <t>绝对收益最大回撤</t>
+  </si>
+  <si>
+    <t>#title#</t>
+  </si>
+  <si>
+    <t>#annual_return#</t>
+  </si>
+  <si>
+    <t>年化双边换手</t>
     <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>开始日期</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>结束日期</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>收益率</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>年化收益率</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>超额收益率（几何）</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>绝对收益最大回撤</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>夏普比率</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>超额夏普比率</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>#title#</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>#start_date#</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>#end_date#</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>#returns#</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>#max_drawdown#</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>#sharpe#</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>#excess_sharpe#</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>#geometric_excess_return#</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>#geometric_excess_drawdown#</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>#annual_return#</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>超额最大回撤持续时间</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>最大回撤持续时间</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>收益最大回撤</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>超额最大回撤（几何）</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>超额最大回撤（几何）</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>#alpha#</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>#beta#</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>阿尔法</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>贝塔</t>
-    <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -657,13 +573,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="5">
-    <numFmt numFmtId="176" formatCode="yyyy/m/d;@"/>
+    <numFmt numFmtId="176" formatCode="0.00_ "/>
     <numFmt numFmtId="177" formatCode="0.000_ "/>
-    <numFmt numFmtId="178" formatCode="0.00_ "/>
+    <numFmt numFmtId="178" formatCode="0_ "/>
     <numFmt numFmtId="179" formatCode="0_);[Red]\(0\)"/>
-    <numFmt numFmtId="180" formatCode="0_ "/>
+    <numFmt numFmtId="180" formatCode="yyyy/m/d;@"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -676,12 +592,6 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
@@ -850,88 +760,88 @@
   </cellStyleXfs>
   <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="4" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="4" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="4" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="4" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="4" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="3" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="10" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="178" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="176" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="180" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="-3522966690757464237" xfId="1" xr:uid="{00000000-0005-0000-0000-00000B000000}"/>
-    <cellStyle name="-4237263631367923067" xfId="2" xr:uid="{00000000-0005-0000-0000-00002E000000}"/>
+    <cellStyle name="-3522966690757464237" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="-4237263631367923067" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
     <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -951,15 +861,8 @@
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="zh-CN"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
+  <c:roundedCorners val="1"/>
+  <c:style val="2"/>
   <c:chart>
     <c:title>
       <c:tx>
@@ -968,7 +871,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr defTabSz="914400">
-              <a:defRPr lang="zh-CN" sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:defRPr lang="zh-CN" sz="1400" b="0" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -992,29 +895,9 @@
         <a:noFill/>
         <a:ln>
           <a:noFill/>
+          <a:prstDash val="solid"/>
         </a:ln>
-        <a:effectLst/>
       </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr defTabSz="914400">
-            <a:defRPr lang="zh-CN" sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="zh-CN"/>
-        </a:p>
-      </c:txPr>
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
@@ -1041,9 +924,9 @@
               <a:solidFill>
                 <a:schemeClr val="accent1"/>
               </a:solidFill>
+              <a:prstDash val="solid"/>
               <a:round/>
             </a:ln>
-            <a:effectLst/>
           </c:spPr>
           <c:marker>
             <c:symbol val="none"/>
@@ -1074,7 +957,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-612A-4FB7-B5FF-52379480CFB5}"/>
+              <c16:uniqueId val="{00000000-5FB6-9843-A355-3F73DC8A3A2D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1097,9 +980,9 @@
               <a:solidFill>
                 <a:schemeClr val="accent2"/>
               </a:solidFill>
+              <a:prstDash val="solid"/>
               <a:round/>
             </a:ln>
-            <a:effectLst/>
           </c:spPr>
           <c:marker>
             <c:symbol val="none"/>
@@ -1130,7 +1013,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-612A-4FB7-B5FF-52379480CFB5}"/>
+              <c16:uniqueId val="{00000001-5FB6-9843-A355-3F73DC8A3A2D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1153,9 +1036,9 @@
               <a:solidFill>
                 <a:schemeClr val="accent3"/>
               </a:solidFill>
+              <a:prstDash val="solid"/>
               <a:round/>
             </a:ln>
-            <a:effectLst/>
           </c:spPr>
           <c:marker>
             <c:symbol val="none"/>
@@ -1186,7 +1069,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-612A-4FB7-B5FF-52379480CFB5}"/>
+              <c16:uniqueId val="{00000002-5FB6-9843-A355-3F73DC8A3A2D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1202,7 +1085,7 @@
         <c:axId val="101121013"/>
         <c:axId val="195469628"/>
       </c:lineChart>
-      <c:dateAx>
+      <c:catAx>
         <c:axId val="101121013"/>
         <c:scaling>
           <c:orientation val="minMax"/>
@@ -1222,16 +1105,16 @@
                 <a:lumOff val="85000"/>
               </a:schemeClr>
             </a:solidFill>
+            <a:prstDash val="solid"/>
             <a:round/>
           </a:ln>
-          <a:effectLst/>
         </c:spPr>
         <c:txPr>
           <a:bodyPr rot="0" spcFirstLastPara="0" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1" forceAA="0"/>
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr lang="zh-CN" sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr lang="zh-CN" sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -1248,10 +1131,11 @@
         </c:txPr>
         <c:crossAx val="195469628"/>
         <c:crosses val="autoZero"/>
-        <c:auto val="0"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
-        <c:baseTimeUnit val="days"/>
-      </c:dateAx>
+        <c:noMultiLvlLbl val="1"/>
+      </c:catAx>
       <c:valAx>
         <c:axId val="195469628"/>
         <c:scaling>
@@ -1268,9 +1152,9 @@
                   <a:lumOff val="85000"/>
                 </a:schemeClr>
               </a:solidFill>
+              <a:prstDash val="solid"/>
               <a:round/>
             </a:ln>
-            <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
         <c:numFmt formatCode="0.00%" sourceLinked="1"/>
@@ -1281,15 +1165,15 @@
           <a:noFill/>
           <a:ln>
             <a:noFill/>
+            <a:prstDash val="solid"/>
           </a:ln>
-          <a:effectLst/>
         </c:spPr>
         <c:txPr>
           <a:bodyPr rot="-60000000" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr lang="zh-CN" sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr lang="zh-CN" sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -1308,13 +1192,6 @@
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
     </c:plotArea>
     <c:legend>
       <c:legendPos val="b"/>
@@ -1333,15 +1210,15 @@
         <a:noFill/>
         <a:ln>
           <a:noFill/>
+          <a:prstDash val="solid"/>
         </a:ln>
-        <a:effectLst/>
       </c:spPr>
       <c:txPr>
         <a:bodyPr rot="0" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr lang="zh-CN" sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+            <a:defRPr lang="zh-CN" sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="65000"/>
@@ -1359,7 +1236,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
+    <c:showDLblsOverMax val="1"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1372,582 +1249,16 @@
           <a:lumOff val="85000"/>
         </a:schemeClr>
       </a:solidFill>
+      <a:prstDash val="solid"/>
       <a:round/>
     </a:ln>
-    <a:effectLst/>
   </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr lang="zh-CN"/>
-      </a:pPr>
-      <a:endParaRPr lang="zh-CN"/>
-    </a:p>
-  </c:txPr>
   <c:printSettings>
     <c:headerFooter/>
     <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
-</file>
-
-<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
-</file>
-
-<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-    </cs:spPr>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-    </cs:spPr>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="28575" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="65000"/>
-          <a:lumOff val="35000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="75000"/>
-            <a:lumOff val="25000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:prstDash val="sysDot"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:wall>
-</cs:chartStyle>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1967,10 +1278,10 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="3" name="图表 2">
+        <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2277,14 +1588,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B52"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="20" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="34" style="2" customWidth="1"/>
     <col min="2" max="2" width="46.5" style="2" customWidth="1"/>
-    <col min="3" max="16384" width="8.875" style="2"/>
+    <col min="3" max="3" width="8.83203125" style="2" customWidth="1"/>
+    <col min="4" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:2" ht="20" customHeight="1">
       <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
@@ -2292,7 +1604,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:2" ht="20" customHeight="1">
       <c r="A2" s="13" t="s">
         <v>2</v>
       </c>
@@ -2300,7 +1612,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:2" ht="20" customHeight="1">
       <c r="A3" s="13" t="s">
         <v>4</v>
       </c>
@@ -2308,7 +1620,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:2" ht="20" customHeight="1">
       <c r="A4" s="13" t="s">
         <v>6</v>
       </c>
@@ -2316,7 +1628,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:2" ht="20" customHeight="1">
       <c r="A5" s="13" t="s">
         <v>8</v>
       </c>
@@ -2324,7 +1636,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:2" ht="20" customHeight="1">
       <c r="A6" s="13" t="s">
         <v>10</v>
       </c>
@@ -2332,7 +1644,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:2" ht="20" customHeight="1">
       <c r="A7" s="13" t="s">
         <v>12</v>
       </c>
@@ -2340,7 +1652,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:2" ht="20" customHeight="1">
       <c r="A8" s="14" t="s">
         <v>14</v>
       </c>
@@ -2348,7 +1660,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:2" ht="20" customHeight="1">
       <c r="A9" s="14" t="s">
         <v>16</v>
       </c>
@@ -2356,7 +1668,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:2" ht="20" customHeight="1">
       <c r="A10" s="14" t="s">
         <v>18</v>
       </c>
@@ -2364,7 +1676,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:2" ht="20" customHeight="1">
       <c r="A11" s="14" t="s">
         <v>20</v>
       </c>
@@ -2372,7 +1684,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:2" ht="20" customHeight="1">
       <c r="A12" s="14" t="s">
         <v>22</v>
       </c>
@@ -2380,15 +1692,15 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:2" ht="20" customHeight="1">
       <c r="A13" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="B13" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="B13" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:2" ht="20" customHeight="1">
       <c r="A14" s="14" t="s">
         <v>26</v>
       </c>
@@ -2396,7 +1708,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:2" ht="20" customHeight="1">
       <c r="A15" s="14" t="s">
         <v>28</v>
       </c>
@@ -2404,7 +1716,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:2" ht="20" customHeight="1">
       <c r="A16" s="13" t="s">
         <v>30</v>
       </c>
@@ -2412,7 +1724,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:2" ht="20" customHeight="1">
       <c r="A17" s="13" t="s">
         <v>32</v>
       </c>
@@ -2420,7 +1732,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:2" ht="20" customHeight="1">
       <c r="A18" s="13" t="s">
         <v>34</v>
       </c>
@@ -2428,7 +1740,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:2" ht="20" customHeight="1">
       <c r="A19" s="13" t="s">
         <v>36</v>
       </c>
@@ -2436,7 +1748,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:2" ht="20" customHeight="1">
       <c r="A20" s="13" t="s">
         <v>38</v>
       </c>
@@ -2444,7 +1756,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:2" ht="20" customHeight="1">
       <c r="A21" s="13" t="s">
         <v>40</v>
       </c>
@@ -2452,7 +1764,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:2" ht="20" customHeight="1">
       <c r="A22" s="13" t="s">
         <v>42</v>
       </c>
@@ -2460,7 +1772,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:2" ht="20" customHeight="1">
       <c r="A23" s="13" t="s">
         <v>44</v>
       </c>
@@ -2468,7 +1780,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:2" ht="20" customHeight="1">
       <c r="A24" s="13" t="s">
         <v>46</v>
       </c>
@@ -2476,7 +1788,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:2" ht="20" customHeight="1">
       <c r="A25" s="13" t="s">
         <v>48</v>
       </c>
@@ -2484,7 +1796,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:2" ht="20" customHeight="1">
       <c r="A26" s="13" t="s">
         <v>50</v>
       </c>
@@ -2492,7 +1804,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:2" ht="20" customHeight="1">
       <c r="A27" s="13" t="s">
         <v>52</v>
       </c>
@@ -2500,7 +1812,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:2" ht="20" customHeight="1">
       <c r="A28" s="13" t="s">
         <v>54</v>
       </c>
@@ -2508,7 +1820,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:2" ht="20" customHeight="1">
       <c r="A29" s="13" t="s">
         <v>56</v>
       </c>
@@ -2516,7 +1828,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:2" ht="20" customHeight="1">
       <c r="A30" s="14" t="s">
         <v>58</v>
       </c>
@@ -2524,7 +1836,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:2" ht="20" customHeight="1">
       <c r="A31" s="14" t="s">
         <v>60</v>
       </c>
@@ -2532,7 +1844,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:2" ht="20" customHeight="1">
       <c r="A32" s="14" t="s">
         <v>62</v>
       </c>
@@ -2540,7 +1852,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="33" spans="1:2" ht="20" customHeight="1">
       <c r="A33" s="14" t="s">
         <v>64</v>
       </c>
@@ -2548,7 +1860,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="34" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="34" spans="1:2" ht="20" customHeight="1">
       <c r="A34" s="14" t="s">
         <v>66</v>
       </c>
@@ -2556,7 +1868,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="35" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="35" spans="1:2" ht="20" customHeight="1">
       <c r="A35" s="14" t="s">
         <v>68</v>
       </c>
@@ -2564,7 +1876,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="36" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="36" spans="1:2" ht="20" customHeight="1">
       <c r="A36" s="14" t="s">
         <v>70</v>
       </c>
@@ -2572,7 +1884,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="37" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="37" spans="1:2" ht="20" customHeight="1">
       <c r="A37" s="14" t="s">
         <v>72</v>
       </c>
@@ -2580,7 +1892,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="38" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="38" spans="1:2" ht="20" customHeight="1">
       <c r="A38" s="14" t="s">
         <v>74</v>
       </c>
@@ -2588,7 +1900,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="39" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="39" spans="1:2" ht="20" customHeight="1">
       <c r="A39" s="14" t="s">
         <v>76</v>
       </c>
@@ -2596,7 +1908,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="40" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="40" spans="1:2" ht="20" customHeight="1">
       <c r="A40" s="14" t="s">
         <v>78</v>
       </c>
@@ -2604,7 +1916,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="41" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="41" spans="1:2" ht="20" customHeight="1">
       <c r="A41" s="13" t="s">
         <v>80</v>
       </c>
@@ -2612,7 +1924,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="42" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="42" spans="1:2" ht="20" customHeight="1">
       <c r="A42" s="13" t="s">
         <v>82</v>
       </c>
@@ -2620,7 +1932,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="43" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="43" spans="1:2" ht="20" customHeight="1">
       <c r="A43" s="13" t="s">
         <v>84</v>
       </c>
@@ -2628,7 +1940,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="44" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="44" spans="1:2" ht="20" customHeight="1">
       <c r="A44" s="13" t="s">
         <v>86</v>
       </c>
@@ -2636,7 +1948,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="45" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="45" spans="1:2" ht="20" customHeight="1">
       <c r="A45" s="13" t="s">
         <v>88</v>
       </c>
@@ -2644,7 +1956,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="46" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="46" spans="1:2" ht="20" customHeight="1">
       <c r="A46" s="13" t="s">
         <v>90</v>
       </c>
@@ -2652,7 +1964,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="47" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="47" spans="1:2" ht="20" customHeight="1">
       <c r="A47" s="13" t="s">
         <v>92</v>
       </c>
@@ -2660,7 +1972,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="48" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="48" spans="1:2" ht="20" customHeight="1">
       <c r="A48" s="13" t="s">
         <v>94</v>
       </c>
@@ -2668,7 +1980,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="49" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="49" spans="1:2" ht="20" customHeight="1">
       <c r="A49" s="13" t="s">
         <v>96</v>
       </c>
@@ -2676,7 +1988,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="50" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="50" spans="1:2" ht="20" customHeight="1">
       <c r="A50" s="13" t="s">
         <v>98</v>
       </c>
@@ -2684,7 +1996,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="51" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="51" spans="1:2" ht="20" customHeight="1">
       <c r="A51" s="13" t="s">
         <v>100</v>
       </c>
@@ -2692,7 +2004,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="52" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="52" spans="1:2" ht="20" customHeight="1">
       <c r="A52" s="15" t="s">
         <v>102</v>
       </c>
@@ -2701,7 +2013,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -2709,15 +2021,18 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:R2"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="18.75" x14ac:dyDescent="0.15"/>
+  <dimension ref="A1:S2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="17"/>
   <cols>
-    <col min="1" max="1" width="12.625" style="2" customWidth="1"/>
-    <col min="2" max="18" width="24.625" style="2" customWidth="1"/>
-    <col min="19" max="16384" width="10.875" style="2"/>
+    <col min="1" max="1" width="12.6640625" style="2" customWidth="1"/>
+    <col min="2" max="12" width="24.6640625" style="2" customWidth="1"/>
+    <col min="13" max="14" width="13" customWidth="1"/>
+    <col min="15" max="18" width="24.6640625" style="2" customWidth="1"/>
+    <col min="19" max="19" width="10.83203125" style="2" customWidth="1"/>
+    <col min="20" max="16384" width="10.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:19" ht="20" customHeight="1">
       <c r="A1" s="21" t="s">
         <v>104</v>
       </c>
@@ -2731,81 +2046,84 @@
         <v>106</v>
       </c>
       <c r="E1" s="21" t="s">
-        <v>189</v>
+        <v>107</v>
       </c>
       <c r="F1" s="21" t="s">
-        <v>188</v>
+        <v>108</v>
       </c>
       <c r="G1" s="21" t="s">
-        <v>190</v>
+        <v>109</v>
       </c>
       <c r="H1" s="21" t="s">
-        <v>187</v>
+        <v>110</v>
       </c>
       <c r="I1" s="21" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="J1" s="21" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="K1" s="21" t="s">
         <v>32</v>
       </c>
       <c r="L1" s="21" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="M1" s="21" t="s">
         <v>68</v>
       </c>
       <c r="N1" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="O1" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="O1" s="21" t="s">
-        <v>110</v>
-      </c>
       <c r="P1" s="21" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="Q1" s="21" t="s">
-        <v>194</v>
+        <v>115</v>
       </c>
       <c r="R1" s="21" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="2" spans="1:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+        <v>64</v>
+      </c>
+      <c r="S1" s="21" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" ht="20" customHeight="1">
       <c r="A2" s="16" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="E2" s="17" t="s">
         <v>39</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="H2" s="19" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="I2" s="17" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="J2" s="17" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="K2" s="20" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="L2" s="20" t="s">
         <v>71</v>
@@ -2813,24 +2131,27 @@
       <c r="M2" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="N2" s="17" t="s">
-        <v>122</v>
+      <c r="N2" s="20" t="s">
+        <v>25</v>
       </c>
       <c r="O2" s="17" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="P2" s="17" t="s">
+        <v>127</v>
+      </c>
+      <c r="Q2" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="Q2" s="17" t="s">
-        <v>192</v>
-      </c>
       <c r="R2" s="17" t="s">
-        <v>193</v>
+        <v>65</v>
+      </c>
+      <c r="S2" s="17" t="s">
+        <v>67</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2838,101 +2159,102 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:N2"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="18" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="1" width="10.875" style="22" customWidth="1"/>
-    <col min="2" max="14" width="16.625" style="22" customWidth="1"/>
-    <col min="15" max="16384" width="10.875" style="22"/>
+    <col min="1" max="1" width="10.83203125" style="22" customWidth="1"/>
+    <col min="2" max="14" width="16.6640625" style="22" customWidth="1"/>
+    <col min="15" max="15" width="10.83203125" style="22" customWidth="1"/>
+    <col min="16" max="16384" width="10.83203125" style="22"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:14" ht="20" customHeight="1">
       <c r="A1" s="21"/>
       <c r="B1" s="21" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C1" s="21" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="D1" s="21" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="E1" s="21" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="F1" s="21" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="G1" s="21" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="H1" s="21" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="I1" s="21" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="J1" s="21" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="K1" s="21" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="L1" s="21" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="M1" s="21" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="N1" s="21" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="20" customHeight="1">
       <c r="A2" s="22" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="F2" s="23" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="G2" s="23" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="H2" s="23" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="I2" s="23" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="J2" s="23" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="K2" s="23" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="L2" s="23" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="M2" s="23" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="N2" s="23" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2940,101 +2262,102 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:N2"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="18" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="1" width="10.875" style="22" customWidth="1"/>
-    <col min="2" max="14" width="16.625" style="22" customWidth="1"/>
-    <col min="15" max="16384" width="10.875" style="22"/>
+    <col min="1" max="1" width="10.83203125" style="22" customWidth="1"/>
+    <col min="2" max="14" width="16.6640625" style="22" customWidth="1"/>
+    <col min="15" max="15" width="10.83203125" style="22" customWidth="1"/>
+    <col min="16" max="16384" width="10.83203125" style="22"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:14" ht="20" customHeight="1">
       <c r="A1" s="21"/>
       <c r="B1" s="21" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C1" s="21" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="D1" s="21" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="E1" s="21" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="F1" s="21" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="G1" s="21" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="H1" s="21" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="I1" s="21" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="J1" s="21" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="K1" s="21" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="L1" s="21" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="M1" s="21" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="N1" s="21" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="20" customHeight="1">
       <c r="A2" s="22" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="F2" s="23" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="G2" s="23" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="H2" s="23" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="I2" s="23" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="J2" s="23" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="K2" s="23" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="L2" s="23" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="M2" s="23" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="N2" s="23" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -3042,158 +2365,160 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultColWidth="9.25" defaultRowHeight="18" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="2" width="14.625" style="22" customWidth="1"/>
-    <col min="3" max="9" width="10.625" style="22" customWidth="1"/>
-    <col min="10" max="16384" width="9.25" style="22"/>
+    <col min="1" max="2" width="14.6640625" style="22" customWidth="1"/>
+    <col min="3" max="9" width="10.6640625" style="22" customWidth="1"/>
+    <col min="10" max="10" width="9.1640625" style="22" customWidth="1"/>
+    <col min="11" max="16384" width="9.1640625" style="22"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:9">
       <c r="A1" s="21" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="B1" s="21" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="C1" s="21" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D1" s="21" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="E1" s="21" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="F1" s="26" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="G1" s="26" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="H1" s="26" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="I1" s="21" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.15">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" s="24" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="B2" s="25" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="F2" s="23" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="G2" s="23" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="H2" s="23" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="I2" s="23" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F84C164A-7D84-4A32-8840-7EDA24C0A2B6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:P2"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="18.75" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="17"/>
   <cols>
-    <col min="1" max="1" width="20.625" style="2" customWidth="1"/>
-    <col min="2" max="5" width="24.625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="24.625" style="17" customWidth="1"/>
-    <col min="7" max="7" width="24.625" style="2" customWidth="1"/>
-    <col min="8" max="8" width="24.625" style="17" customWidth="1"/>
-    <col min="9" max="10" width="24.625" style="2" customWidth="1"/>
-    <col min="11" max="11" width="14.375" style="2" customWidth="1"/>
-    <col min="12" max="12" width="16.875" style="2" customWidth="1"/>
+    <col min="1" max="1" width="20.6640625" style="2" customWidth="1"/>
+    <col min="2" max="5" width="24.6640625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="24.6640625" style="17" customWidth="1"/>
+    <col min="7" max="7" width="24.6640625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="24.6640625" style="17" customWidth="1"/>
+    <col min="9" max="10" width="24.6640625" style="2" customWidth="1"/>
+    <col min="11" max="11" width="14.33203125" style="2" customWidth="1"/>
+    <col min="12" max="12" width="16.83203125" style="2" customWidth="1"/>
     <col min="13" max="13" width="16.5" style="2" customWidth="1"/>
     <col min="14" max="14" width="21" style="2" customWidth="1"/>
-    <col min="15" max="15" width="22.375" style="2" customWidth="1"/>
-    <col min="16" max="16384" width="10.875" style="2"/>
+    <col min="15" max="15" width="22.33203125" style="2" customWidth="1"/>
+    <col min="16" max="16" width="10.83203125" style="2" customWidth="1"/>
+    <col min="17" max="16384" width="10.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:16" ht="20" customHeight="1">
       <c r="A1" s="21" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="B1" s="21" t="s">
-        <v>169</v>
+        <v>2</v>
       </c>
       <c r="C1" s="21" t="s">
-        <v>170</v>
+        <v>4</v>
       </c>
       <c r="D1" s="21" t="s">
-        <v>171</v>
+        <v>18</v>
       </c>
       <c r="E1" s="21" t="s">
-        <v>172</v>
+        <v>20</v>
       </c>
       <c r="F1" s="26" t="s">
+        <v>106</v>
+      </c>
+      <c r="G1" s="21" t="s">
         <v>173</v>
       </c>
-      <c r="G1" s="21" t="s">
+      <c r="H1" s="26" t="s">
+        <v>109</v>
+      </c>
+      <c r="I1" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="J1" s="21" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" ht="20" customHeight="1">
+      <c r="A2" s="16" t="s">
         <v>174</v>
       </c>
-      <c r="H1" s="26" t="s">
-        <v>191</v>
-      </c>
-      <c r="I1" s="21" t="s">
+      <c r="B2" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>117</v>
+      </c>
+      <c r="E2" s="17" t="s">
         <v>175</v>
       </c>
-      <c r="J1" s="21" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="2" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="16" t="s">
-        <v>177</v>
-      </c>
-      <c r="B2" s="17" t="s">
-        <v>178</v>
-      </c>
-      <c r="C2" s="17" t="s">
-        <v>179</v>
-      </c>
-      <c r="D2" s="17" t="s">
-        <v>180</v>
-      </c>
-      <c r="E2" s="17" t="s">
-        <v>186</v>
-      </c>
       <c r="F2" s="17" t="s">
-        <v>184</v>
+        <v>119</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>181</v>
+        <v>39</v>
       </c>
       <c r="H2" s="17" t="s">
-        <v>185</v>
+        <v>121</v>
       </c>
       <c r="I2" s="17" t="s">
-        <v>182</v>
+        <v>33</v>
       </c>
       <c r="J2" s="17" t="s">
-        <v>183</v>
+        <v>71</v>
       </c>
       <c r="K2" s="20"/>
       <c r="L2" s="20"/>

</xml_diff>